<commit_message>
docs(import): record Jeroen fase1 decisions and Tim Couwenberg email write.
LEOXX address overwrite refused; brand 140480 got atelier@timcouwenberg.com.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/import/mdu2026-fair-compleet/oordeel/fase1-oordeel-jeroen.xlsx
+++ b/docs/import/mdu2026-fair-compleet/oordeel/fase1-oordeel-jeroen.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26940" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAMENVATTING" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEL_matched" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -29,22 +28,24 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid"/>
     </fill>
   </fills>
   <borders count="1">
@@ -59,14 +60,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -430,9 +430,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="63.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>MDU 2026 fase 1 — merken (prepare 2026-09-10)</t>
@@ -565,60 +568,71 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="6.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="9.6640625" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="23.83203125" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="31.1640625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="40.33203125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="21.1640625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="10.5" bestFit="1" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>zaak_id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>merk</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>veld</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>nu_in_DB</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>voorstel_bron</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>reden_machine</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>risico</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>BESLIST</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>TOELICHTING</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>beslist_door</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>beslist_op</t>
         </is>
@@ -660,14 +674,26 @@
           <t>HOOG — zwakkere bron zou sterkere overschrijven</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NIET</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>voorstel: NIET (laten staan)</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+          <t>Akkoord voorstel: laten staan (zwakkere bron niet overschrijven)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Jeroen</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -705,14 +731,26 @@
           <t>HOOG — zwakkere bron zou sterkere overschrijven</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>NIET</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>voorstel: NIET (laten staan)</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+          <t>Akkoord voorstel: laten staan (zwakkere bron niet overschrijven)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Jeroen</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -750,14 +788,26 @@
           <t>HOOG — zwakkere bron zou sterkere overschrijven</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NIET</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>voorstel: NIET (laten staan)</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+          <t>Akkoord voorstel: laten staan (zwakkere bron niet overschrijven)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Jeroen</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -775,7 +825,6 @@
           <t>email</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>atelier@timcouwenberg.com</t>
@@ -791,14 +840,26 @@
           <t>laag — leeg veld vullen</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>WEL</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>voorstel: WEL vullen</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+          <t>Akkoord voorstel: leeg veld vullen</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Jeroen</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -812,30 +873,37 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="37" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="6.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="70.6640625" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="38" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>brand_name</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>stand</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>reden</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>notitie</t>
         </is>
@@ -847,7 +915,6 @@
           <t>BAGUETTE STUDIO</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>B25</t>
@@ -865,8 +932,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>A12</t>
@@ -884,8 +949,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>O01</t>
@@ -930,8 +993,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>NNP01</t>
@@ -954,7 +1015,6 @@
           <t>Tamar Alon</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>E28</t>
@@ -977,7 +1037,6 @@
           <t>Carmen Enríquez</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>C12</t>
@@ -995,8 +1054,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>F09</t>
@@ -1019,7 +1076,6 @@
           <t>Diana Kusyová</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>C15</t>
@@ -1042,7 +1098,6 @@
           <t>Observology</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>A18</t>
@@ -1065,7 +1120,6 @@
           <t>Maëlys Venkiah</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>A03</t>
@@ -1110,8 +1164,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>B01</t>
@@ -1156,8 +1208,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>D01</t>
@@ -1202,8 +1252,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>B24</t>
@@ -1221,8 +1269,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>F17</t>
@@ -1251,30 +1297,37 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E106"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="33.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="8" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="36" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="89.5" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>brand_name</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>brand_id</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>al_exposant</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>reden</t>
         </is>

</xml_diff>